<commit_message>
APEX 35 : salle JEV prospectif, retours TypeSafe, corrections graphiques premium
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkwQ8QV1wk6UyfQvHD3u4J
</commit_message>
<xml_diff>
--- a/typesafe-reporting/sortie/JEV_Risque_Prospectif_demo.xlsx
+++ b/typesafe-reporting/sortie/JEV_Risque_Prospectif_demo.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="316">
   <si>
     <t>JEV · MOTEUR DE JUGEMENT PROBABILISTE ET D'ÉVOLUTION DU RISQUE</t>
   </si>
@@ -296,9 +296,6 @@
     <t>Régularisation complète des impayés (retour en Sain)</t>
   </si>
   <si>
-    <t>nature de l'entité incertaine (0.49)</t>
-  </si>
-  <si>
     <t>MARKOV · Markov mensuel Commercial (MLE sur 17 transitions) · N = 16 337 · Historique = 18 mois · Confiance = faible | EXPERT ×2.00 Client injoignable (TypeSafe)</t>
   </si>
   <si>
@@ -398,7 +395,7 @@
     <t>Santé / décès</t>
   </si>
   <si>
-    <t>statut incertain (0.40)</t>
+    <t>statut incertain (0.44)</t>
   </si>
   <si>
     <t>MARKOV · Markov mensuel Consumer (MLE sur 17 transitions) · N = 38 478 · Historique = 18 mois · Confiance = faible</t>
@@ -425,7 +422,7 @@
     <t>DIALLO AMADOU</t>
   </si>
   <si>
-    <t>nature de l'entité incertaine (0.45)</t>
+    <t>nature de l'entité incertaine (0.47)</t>
   </si>
   <si>
     <t>MARKOV · Markov mensuel Corporate (MLE sur 17 transitions) · N = 6 689 · Historique = 18 mois · Confiance = faible</t>
@@ -503,7 +500,7 @@
     <t>GIE DES MARAICHERS DE NIAYES</t>
   </si>
   <si>
-    <t>crédibilité incertaine (0.21)</t>
+    <t>crédibilité incertaine (0.31)</t>
   </si>
   <si>
     <t>LD9000019</t>
@@ -512,7 +509,7 @@
     <t>SOCIETE DE TRANSPORT URBAIN DE THIES</t>
   </si>
   <si>
-    <t>motif incertain (0.34)</t>
+    <t>motif incertain (0.36)</t>
   </si>
   <si>
     <t>LD9000006</t>
@@ -554,9 +551,6 @@
     <t>Promesse crédible avant bascule (TypeSafe + code)</t>
   </si>
   <si>
-    <t>statut incertain (0.54)</t>
-  </si>
-  <si>
     <t>MARKOV · Markov mensuel Consumer (MLE sur 17 transitions) · N = 38 478 · Historique = 18 mois · Confiance = faible | EXPERT ×0.75 Promesse crédible avant bascule (TypeSafe + code)</t>
   </si>
   <si>
@@ -564,6 +558,9 @@
   </si>
   <si>
     <t>FALL IBRAHIMA</t>
+  </si>
+  <si>
+    <t>statut incertain (0.37)</t>
   </si>
   <si>
     <t>MARKOV · Markov mensuel Consumer (MLE sur 17 transitions) · N = 38 478 · Historique = 18 mois · Confiance = faible | EXPERT ×0.75 Promesse crédible avant bascule (TypeSafe + code) | EXPERT ×0.70 Incident technique (TypeSafe)</t>
@@ -3751,19 +3748,17 @@
       <c r="P7" s="16">
         <v>0.2142456429720498</v>
       </c>
-      <c r="Q7" s="14" t="s">
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14" t="s">
         <v>91</v>
-      </c>
-      <c r="R7" s="14" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>93</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>94</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>45</v>
@@ -3775,10 +3770,10 @@
         <v>85</v>
       </c>
       <c r="F8" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>95</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>96</v>
       </c>
       <c r="H8" s="16">
         <v>0.6365657247068505</v>
@@ -3809,12 +3804,12 @@
       </c>
       <c r="Q8" s="14"/>
       <c r="R8" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>54</v>
@@ -3829,10 +3824,10 @@
         <v>85</v>
       </c>
       <c r="F9" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>100</v>
       </c>
       <c r="H9" s="16">
         <v>0.6365657247068505</v>
@@ -3863,12 +3858,12 @@
       </c>
       <c r="Q9" s="14"/>
       <c r="R9" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>55</v>
@@ -3883,10 +3878,10 @@
         <v>85</v>
       </c>
       <c r="F10" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>104</v>
       </c>
       <c r="H10" s="16">
         <v>0.6938187099288988</v>
@@ -3917,12 +3912,12 @@
       </c>
       <c r="Q10" s="14"/>
       <c r="R10" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>56</v>
@@ -3937,10 +3932,10 @@
         <v>85</v>
       </c>
       <c r="F11" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="G11" s="14" t="s">
         <v>107</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>108</v>
       </c>
       <c r="H11" s="16">
         <v>0.6365657247068505</v>
@@ -3971,12 +3966,12 @@
       </c>
       <c r="Q11" s="14"/>
       <c r="R11" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>57</v>
@@ -3991,10 +3986,10 @@
         <v>85</v>
       </c>
       <c r="F12" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="G12" s="14" t="s">
         <v>111</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>112</v>
       </c>
       <c r="H12" s="16">
         <v>0.6365657247068505</v>
@@ -4024,18 +4019,18 @@
         <v>0.1701031348772964</v>
       </c>
       <c r="Q12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="R12" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="R12" s="14" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>115</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>116</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>46</v>
@@ -4047,10 +4042,10 @@
         <v>85</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H13" s="16">
         <v>0.6938187099288988</v>
@@ -4065,7 +4060,7 @@
         <v>0.6938187099288988</v>
       </c>
       <c r="L13" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M13" s="13" t="s">
         <v>89</v>
@@ -4081,12 +4076,12 @@
       </c>
       <c r="Q13" s="14"/>
       <c r="R13" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>59</v>
@@ -4101,10 +4096,10 @@
         <v>85</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H14" s="16">
         <v>0.4695200974274228</v>
@@ -4135,12 +4130,12 @@
       </c>
       <c r="Q14" s="14"/>
       <c r="R14" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>60</v>
@@ -4155,10 +4150,10 @@
         <v>85</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H15" s="16">
         <v>0.6365657247068505</v>
@@ -4173,7 +4168,7 @@
         <v>0.6365657247068505</v>
       </c>
       <c r="L15" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M15" s="13" t="s">
         <v>89</v>
@@ -4188,15 +4183,15 @@
         <v>0.1361948349147899</v>
       </c>
       <c r="Q15" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="R15" s="14" t="s">
         <v>125</v>
-      </c>
-      <c r="R15" s="14" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>61</v>
@@ -4211,10 +4206,10 @@
         <v>85</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H16" s="16">
         <v>0.6365657247068505</v>
@@ -4229,7 +4224,7 @@
         <v>0.6365657247068505</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M16" s="13" t="s">
         <v>89</v>
@@ -4245,15 +4240,15 @@
       </c>
       <c r="Q16" s="14"/>
       <c r="R16" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>128</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>129</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>46</v>
@@ -4262,13 +4257,13 @@
         <v>55</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F17" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>100</v>
       </c>
       <c r="H17" s="16">
         <v>0.3999794512425623</v>
@@ -4299,15 +4294,15 @@
       </c>
       <c r="Q17" s="14"/>
       <c r="R17" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>132</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>133</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>47</v>
@@ -4319,10 +4314,10 @@
         <v>85</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H18" s="16">
         <v>0.4695200974274228</v>
@@ -4337,7 +4332,7 @@
         <v>0.4695200974274228</v>
       </c>
       <c r="L18" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M18" s="13" t="s">
         <v>89</v>
@@ -4352,18 +4347,18 @@
         <v>0.04627981914257439</v>
       </c>
       <c r="Q18" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="R18" s="14" t="s">
         <v>134</v>
-      </c>
-      <c r="R18" s="14" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" s="14" t="s">
         <v>136</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>137</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>46</v>
@@ -4372,13 +4367,13 @@
         <v>36</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H19" s="16">
         <v>0.3999794512425623</v>
@@ -4408,18 +4403,18 @@
         <v>0.1505487097213332</v>
       </c>
       <c r="Q19" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R19" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>140</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>141</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>46</v>
@@ -4428,13 +4423,13 @@
         <v>56</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F20" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>143</v>
       </c>
       <c r="H20" s="16">
         <v>0.3999794512425623</v>
@@ -4465,15 +4460,15 @@
       </c>
       <c r="Q20" s="14"/>
       <c r="R20" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B21" s="14" t="s">
         <v>145</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>146</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>46</v>
@@ -4482,13 +4477,13 @@
         <v>49</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H21" s="16">
         <v>0.3999794512425623</v>
@@ -4518,18 +4513,18 @@
         <v>0.1505487097213332</v>
       </c>
       <c r="Q21" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R21" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>147</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>148</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>46</v>
@@ -4538,13 +4533,13 @@
         <v>35</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F22" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>104</v>
       </c>
       <c r="H22" s="16">
         <v>0.3999794512425623</v>
@@ -4575,15 +4570,15 @@
       </c>
       <c r="Q22" s="14"/>
       <c r="R22" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>149</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>150</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>45</v>
@@ -4592,13 +4587,13 @@
         <v>43</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F23" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="G23" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>143</v>
       </c>
       <c r="H23" s="16">
         <v>0.3742985573107679</v>
@@ -4629,15 +4624,15 @@
       </c>
       <c r="Q23" s="14"/>
       <c r="R23" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>153</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>45</v>
@@ -4646,13 +4641,13 @@
         <v>32</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F24" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>104</v>
       </c>
       <c r="H24" s="16">
         <v>0.3742985573107679</v>
@@ -4683,15 +4678,15 @@
       </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" s="14" t="s">
         <v>155</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>156</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>46</v>
@@ -4700,13 +4695,13 @@
         <v>51</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H25" s="16">
         <v>0.3999794512425623</v>
@@ -4721,7 +4716,7 @@
         <v>0.3999794512425623</v>
       </c>
       <c r="L25" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M25" s="13" t="s">
         <v>89</v>
@@ -4736,18 +4731,18 @@
         <v>0.1199748678360338</v>
       </c>
       <c r="Q25" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R25" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B26" s="14" t="s">
         <v>158</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>159</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>46</v>
@@ -4756,13 +4751,13 @@
         <v>56</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H26" s="16">
         <v>0.3999794512425623</v>
@@ -4777,7 +4772,7 @@
         <v>0.3999794512425623</v>
       </c>
       <c r="L26" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M26" s="13" t="s">
         <v>89</v>
@@ -4792,18 +4787,18 @@
         <v>0.1199748678360338</v>
       </c>
       <c r="Q26" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R26" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:18" ht="26" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="14" t="s">
         <v>161</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>162</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>46</v>
@@ -4812,13 +4807,13 @@
         <v>40</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H27" s="16">
         <v>0.3999794512425623</v>
@@ -4833,7 +4828,7 @@
         <v>0.3999794512425623</v>
       </c>
       <c r="L27" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M27" s="13" t="s">
         <v>89</v>
@@ -4848,18 +4843,18 @@
         <v>0.1199748678360338</v>
       </c>
       <c r="Q27" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R27" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>164</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>165</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>47</v>
@@ -4868,13 +4863,13 @@
         <v>58</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F28" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G28" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>100</v>
       </c>
       <c r="H28" s="16">
         <v>0.2391779427856761</v>
@@ -4905,15 +4900,15 @@
       </c>
       <c r="Q28" s="14"/>
       <c r="R28" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29" s="14" t="s">
         <v>167</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>168</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>47</v>
@@ -4925,10 +4920,10 @@
         <v>85</v>
       </c>
       <c r="F29" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G29" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>170</v>
       </c>
       <c r="H29" s="16">
         <v>0.4695200974274228</v>
@@ -4959,15 +4954,15 @@
       </c>
       <c r="Q29" s="14"/>
       <c r="R29" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>172</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>173</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>47</v>
@@ -4979,10 +4974,10 @@
         <v>85</v>
       </c>
       <c r="F30" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G30" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>170</v>
       </c>
       <c r="H30" s="16">
         <v>0.4695200974274228</v>
@@ -5013,15 +5008,15 @@
       </c>
       <c r="Q30" s="14"/>
       <c r="R30" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="B31" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>45</v>
@@ -5030,13 +5025,13 @@
         <v>51</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H31" s="16">
         <v>0.3742985573107679</v>
@@ -5066,18 +5061,18 @@
         <v>0.1057466635317154</v>
       </c>
       <c r="Q31" s="14" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="R31" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>45</v>
@@ -5086,13 +5081,13 @@
         <v>40</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F32" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G32" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>170</v>
       </c>
       <c r="H32" s="16">
         <v>0.3742985573107679</v>
@@ -5122,18 +5117,18 @@
         <v>0.07644789750061205</v>
       </c>
       <c r="Q32" s="14" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="R32" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="B33" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>183</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>48</v>
@@ -5142,7 +5137,7 @@
         <v>37</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F33" s="13" t="s">
         <v>86</v>
@@ -5179,15 +5174,15 @@
       </c>
       <c r="Q33" s="14"/>
       <c r="R33" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="34" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="B34" s="14" t="s">
         <v>185</v>
-      </c>
-      <c r="B34" s="14" t="s">
-        <v>186</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>47</v>
@@ -5196,13 +5191,13 @@
         <v>31</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H34" s="16">
         <v>0.2391779427856761</v>
@@ -5233,15 +5228,15 @@
       </c>
       <c r="Q34" s="14"/>
       <c r="R34" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="B35" s="14" t="s">
         <v>189</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>190</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>47</v>
@@ -5250,13 +5245,13 @@
         <v>52</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F35" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G35" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="G35" s="14" t="s">
-        <v>170</v>
       </c>
       <c r="H35" s="16">
         <v>0.2391779427856761</v>
@@ -5287,15 +5282,15 @@
       </c>
       <c r="Q35" s="14"/>
       <c r="R35" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="B36" s="14" t="s">
         <v>191</v>
-      </c>
-      <c r="B36" s="14" t="s">
-        <v>192</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>48</v>
@@ -5304,13 +5299,13 @@
         <v>36</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H36" s="16">
         <v>0.1012362535335929</v>
@@ -5341,7 +5336,7 @@
       </c>
       <c r="Q36" s="14"/>
       <c r="R36" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -5433,7 +5428,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5449,7 +5444,7 @@
     </row>
     <row r="2" spans="1:12" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5523,7 +5518,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>33</v>
@@ -5561,7 +5556,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B9" s="16">
         <v>0.9709986952715982</v>
@@ -5599,7 +5594,7 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="16">
         <v>0.02052882789145981</v>
@@ -5675,7 +5670,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B12" s="16">
         <v>0.003336140976729591</v>
@@ -5713,7 +5708,7 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -5729,18 +5724,18 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>201</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C17" s="16">
         <v>0.8192360916334702</v>
@@ -5748,7 +5743,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B18" s="16">
         <v>0.3999794512425623</v>
@@ -5756,7 +5751,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B19" s="16">
         <v>0.2938392586863365</v>
@@ -5764,7 +5759,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B20" s="16">
         <v>0.1254173817045714</v>
@@ -5772,7 +5767,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C21" s="16">
         <v>0.814085716050425</v>
@@ -5780,7 +5775,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B22" s="16">
         <v>0.3742985573107679</v>
@@ -5788,7 +5783,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B23" s="16">
         <v>0.2622671673960825</v>
@@ -5796,7 +5791,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B24" s="16">
         <v>0.1775199913435745</v>
@@ -5804,7 +5799,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C25" s="16">
         <v>0.7370114303602556</v>
@@ -5812,7 +5807,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B26" s="16">
         <v>0.3742985573107679</v>
@@ -5820,7 +5815,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B27" s="16">
         <v>0.2622671673960825</v>
@@ -5828,7 +5823,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B28" s="16">
         <v>0.1004457056534052</v>
@@ -5836,7 +5831,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C29" s="16">
         <v>0.7311283466602289</v>
@@ -5844,7 +5839,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B30" s="16">
         <v>0.3999794512425623</v>
@@ -5852,7 +5847,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B31" s="16">
         <v>0.2938392586863365</v>
@@ -5860,7 +5855,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B32" s="16">
         <v>0.03730963673133003</v>
@@ -5868,7 +5863,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C33" s="16">
         <v>0.7103246773769448</v>
@@ -5876,7 +5871,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B34" s="16">
         <v>0.3742985573107679</v>
@@ -5884,7 +5879,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B35" s="16">
         <v>0.2622671673960825</v>
@@ -5892,7 +5887,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B36" s="16">
         <v>0.07375895267009436</v>
@@ -5900,7 +5895,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C37" s="16">
         <v>0.6948417159733646</v>
@@ -5908,7 +5903,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B38" s="16">
         <v>0.3742985573107679</v>
@@ -5916,7 +5911,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B39" s="16">
         <v>0.2622671673960825</v>
@@ -5924,7 +5919,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B40" s="16">
         <v>0.05827599126651417</v>
@@ -5932,7 +5927,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C41" s="16">
         <v>0.6938187099288988</v>
@@ -5940,7 +5935,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B42" s="16">
         <v>0.3999794512425623</v>
@@ -5948,7 +5943,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B43" s="16">
         <v>0.2938392586863365</v>
@@ -5956,7 +5951,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C44" s="16">
         <v>0.6480085314985826</v>
@@ -5964,7 +5959,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B45" s="16">
         <v>0.2391779427856761</v>
@@ -5972,7 +5967,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B46" s="16">
         <v>0.2303421546417468</v>
@@ -5980,7 +5975,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B47" s="16">
         <v>0.1165960672192404</v>
@@ -5988,7 +5983,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B48" s="16">
         <v>0.06189236685191934</v>
@@ -5996,7 +5991,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C49" s="16">
         <v>0.6365657247068505</v>
@@ -6004,7 +5999,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B50" s="16">
         <v>0.3742985573107679</v>
@@ -6012,7 +6007,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B51" s="16">
         <v>0.2622671673960825</v>
@@ -6020,7 +6015,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C52" s="16">
         <v>0.6365657247068505</v>
@@ -6028,7 +6023,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B53" s="16">
         <v>0.3742985573107679</v>
@@ -6036,7 +6031,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B54" s="16">
         <v>0.2622671673960825</v>
@@ -6044,7 +6039,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C55" s="16">
         <v>0.5161076493634182</v>
@@ -6052,7 +6047,7 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B56" s="16">
         <v>0.1199748678360338</v>
@@ -6060,7 +6055,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B57" s="16">
         <v>0.2800045834065285</v>
@@ -6068,7 +6063,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B58" s="16">
         <v>0.116128198120856</v>
@@ -6076,7 +6071,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C59" s="16">
         <v>0.4695200974274228</v>
@@ -6084,7 +6079,7 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B60" s="16">
         <v>0.2391779427856761</v>
@@ -6092,7 +6087,7 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B61" s="16">
         <v>0.2303421546417468</v>
@@ -6100,7 +6095,7 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C62" s="16">
         <v>0.4642644184217922</v>
@@ -6108,7 +6103,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B63" s="16">
         <v>0.1199748678360338</v>
@@ -6116,7 +6111,7 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B64" s="16">
         <v>0.2800045834065285</v>
@@ -6124,7 +6119,7 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B65" s="16">
         <v>0.06428496717922993</v>
@@ -6132,7 +6127,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C66" s="16">
         <v>0.4642644184217922</v>
@@ -6140,7 +6135,7 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B67" s="16">
         <v>0.1199748678360338</v>
@@ -6148,7 +6143,7 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B68" s="16">
         <v>0.2800045834065285</v>
@@ -6156,7 +6151,7 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B69" s="16">
         <v>0.06428496717922993</v>
@@ -6164,7 +6159,7 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C70" s="16">
         <v>0.4642644184217922</v>
@@ -6172,7 +6167,7 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B71" s="16">
         <v>0.1199748678360338</v>
@@ -6180,7 +6175,7 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B72" s="16">
         <v>0.2800045834065285</v>
@@ -6188,7 +6183,7 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B73" s="16">
         <v>0.06428496717922993</v>
@@ -6196,7 +6191,7 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C74" s="16">
         <v>0.4444233036670445</v>
@@ -6204,7 +6199,7 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B75" s="16">
         <v>0.1199748678360338</v>
@@ -6212,7 +6207,7 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B76" s="16">
         <v>0.2800045834065285</v>
@@ -6220,7 +6215,7 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B77" s="16">
         <v>0.04444385242448218</v>
@@ -6228,7 +6223,7 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C78" s="16">
         <v>0.4374653317407829</v>
@@ -6236,7 +6231,7 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B79" s="16">
         <v>0.1361948349147899</v>
@@ -6244,7 +6239,7 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B80" s="16">
         <v>0.238103722395978</v>
@@ -6252,7 +6247,7 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B81" s="16">
         <v>0.063166774430015</v>
@@ -6260,7 +6255,7 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C82" s="16">
         <v>0.4178761786149026</v>
@@ -6268,7 +6263,7 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B83" s="16">
         <v>0.1361948349147899</v>
@@ -6276,7 +6271,7 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B84" s="16">
         <v>0.238103722395978</v>
@@ -6284,7 +6279,7 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B85" s="16">
         <v>0.04357762130413462</v>
@@ -6292,7 +6287,7 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C86" s="16">
         <v>0.3999794512425623</v>
@@ -6300,7 +6295,7 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B87" s="16">
         <v>0.1199748678360338</v>
@@ -6308,7 +6303,7 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B88" s="16">
         <v>0.2800045834065285</v>
@@ -6316,7 +6311,7 @@
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C89" s="16">
         <v>0.3999794512425623</v>
@@ -6324,7 +6319,7 @@
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B90" s="16">
         <v>0.1199748678360338</v>
@@ -6332,7 +6327,7 @@
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B91" s="16">
         <v>0.2800045834065285</v>
@@ -6340,7 +6335,7 @@
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C92" s="16">
         <v>0.3999794512425623</v>
@@ -6348,7 +6343,7 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B93" s="16">
         <v>0.1199748678360338</v>
@@ -6356,7 +6351,7 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B94" s="16">
         <v>0.2800045834065285</v>
@@ -6364,7 +6359,7 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C95" s="16">
         <v>0.3346588931044845</v>
@@ -6372,7 +6367,7 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B96" s="16">
         <v>0.04627981914257438</v>
@@ -6380,7 +6375,7 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B97" s="16">
         <v>0.1928981236431017</v>
@@ -6388,7 +6383,7 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B98" s="16">
         <v>0.09548095031880841</v>
@@ -6396,7 +6391,7 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C99" s="16">
         <v>0.3172523106589988</v>
@@ -6404,7 +6399,7 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B100" s="16">
         <v>0.2391779427856761</v>
@@ -6412,7 +6407,7 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B101" s="16">
         <v>0.2303421546417468</v>
@@ -6420,7 +6415,7 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B102" s="16">
         <v>-0.07054875892585422</v>
@@ -6428,7 +6423,7 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B103" s="16">
         <v>-0.08171902784256968</v>
@@ -6436,7 +6431,7 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" s="10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C104" s="16">
         <v>0.3172523106589988</v>
@@ -6444,7 +6439,7 @@
     </row>
     <row r="105" spans="1:3">
       <c r="A105" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B105" s="16">
         <v>0.2391779427856761</v>
@@ -6452,7 +6447,7 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B106" s="16">
         <v>0.2303421546417468</v>
@@ -6460,7 +6455,7 @@
     </row>
     <row r="107" spans="1:3">
       <c r="A107" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B107" s="16">
         <v>-0.07054875892585422</v>
@@ -6468,7 +6463,7 @@
     </row>
     <row r="108" spans="1:3">
       <c r="A108" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B108" s="16">
         <v>-0.08171902784256968</v>
@@ -6476,7 +6471,7 @@
     </row>
     <row r="109" spans="1:3">
       <c r="A109" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C109" s="16">
         <v>0.3097043950478826</v>
@@ -6484,7 +6479,7 @@
     </row>
     <row r="110" spans="1:3">
       <c r="A110" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B110" s="16">
         <v>0.1361948349147899</v>
@@ -6492,7 +6487,7 @@
     </row>
     <row r="111" spans="1:3">
       <c r="A111" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B111" s="16">
         <v>0.238103722395978</v>
@@ -6500,7 +6495,7 @@
     </row>
     <row r="112" spans="1:3">
       <c r="A112" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B112" s="16">
         <v>-0.06459416226288534</v>
@@ -6508,7 +6503,7 @@
     </row>
     <row r="113" spans="1:3">
       <c r="A113" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C113" s="16">
         <v>0.2389987671089147</v>
@@ -6516,7 +6511,7 @@
     </row>
     <row r="114" spans="1:3">
       <c r="A114" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B114" s="16">
         <v>0.1361948349147899</v>
@@ -6524,7 +6519,7 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B115" s="16">
         <v>0.238103722395978</v>
@@ -6532,7 +6527,7 @@
     </row>
     <row r="116" spans="1:3">
       <c r="A116" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B116" s="16">
         <v>-0.06459416226288534</v>
@@ -6540,7 +6535,7 @@
     </row>
     <row r="117" spans="1:3">
       <c r="A117" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B117" s="16">
         <v>-0.07070562793896792</v>
@@ -6548,7 +6543,7 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C118" s="16">
         <v>0.1838592821635703</v>
@@ -6556,7 +6551,7 @@
     </row>
     <row r="119" spans="1:3">
       <c r="A119" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B119" s="16">
         <v>0.0305385165990613</v>
@@ -6564,7 +6559,7 @@
     </row>
     <row r="120" spans="1:3">
       <c r="A120" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B120" s="16">
         <v>0.07069773693453164</v>
@@ -6572,7 +6567,7 @@
     </row>
     <row r="121" spans="1:3">
       <c r="A121" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B121" s="16">
         <v>0.08262302862997731</v>
@@ -6580,7 +6575,7 @@
     </row>
     <row r="122" spans="1:3">
       <c r="A122" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C122" s="16">
         <v>0.1803664638837456</v>
@@ -6588,7 +6583,7 @@
     </row>
     <row r="123" spans="1:3">
       <c r="A123" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B123" s="16">
         <v>0.04627981914257438</v>
@@ -6596,7 +6591,7 @@
     </row>
     <row r="124" spans="1:3">
       <c r="A124" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B124" s="16">
         <v>0.1928981236431017</v>
@@ -6604,7 +6599,7 @@
     </row>
     <row r="125" spans="1:3">
       <c r="A125" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B125" s="16">
         <v>-0.0588114789019305</v>
@@ -6612,7 +6607,7 @@
     </row>
     <row r="126" spans="1:3">
       <c r="A126" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C126" s="16">
         <v>0.1416626455221195</v>
@@ -6620,7 +6615,7 @@
     </row>
     <row r="127" spans="1:3">
       <c r="A127" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B127" s="16">
         <v>0.04627981914257438</v>
@@ -6628,7 +6623,7 @@
     </row>
     <row r="128" spans="1:3">
       <c r="A128" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B128" s="16">
         <v>0.1928981236431017</v>
@@ -6636,7 +6631,7 @@
     </row>
     <row r="129" spans="1:3">
       <c r="A129" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B129" s="16">
         <v>-0.04838619102475597</v>
@@ -6644,7 +6639,7 @@
     </row>
     <row r="130" spans="1:3">
       <c r="A130" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B130" s="16">
         <v>-0.04912910623880062</v>
@@ -6652,7 +6647,7 @@
     </row>
     <row r="131" spans="1:3">
       <c r="A131" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C131" s="16">
         <v>0.0778987341502909</v>
@@ -6660,7 +6655,7 @@
     </row>
     <row r="132" spans="1:3">
       <c r="A132" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B132" s="16">
         <v>0.0305385165990613</v>
@@ -6668,7 +6663,7 @@
     </row>
     <row r="133" spans="1:3">
       <c r="A133" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B133" s="16">
         <v>0.07069773693453164</v>
@@ -6676,7 +6671,7 @@
     </row>
     <row r="134" spans="1:3">
       <c r="A134" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B134" s="16">
         <v>-0.02333751938330204</v>
@@ -6729,7 +6724,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6746,7 +6741,7 @@
     </row>
     <row r="2" spans="1:13" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6810,40 +6805,40 @@
         <v>30</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="G6" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>254</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>255</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>78</v>
       </c>
       <c r="K6" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="L6" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="M6" s="12" t="s">
         <v>257</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="26" customHeight="1">
@@ -6878,13 +6873,13 @@
         <v>89</v>
       </c>
       <c r="K7" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="M7" s="14" t="s">
         <v>259</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="26" customHeight="1">
@@ -6919,13 +6914,13 @@
         <v>89</v>
       </c>
       <c r="K8" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="M8" s="14" t="s">
         <v>259</v>
-      </c>
-      <c r="L8" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="M8" s="14" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="26" customHeight="1">
@@ -6960,13 +6955,13 @@
         <v>89</v>
       </c>
       <c r="K9" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="M9" s="14" t="s">
         <v>259</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="26" customHeight="1">
@@ -7001,13 +6996,13 @@
         <v>89</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>85</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -7054,7 +7049,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7067,7 +7062,7 @@
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7116,31 +7111,31 @@
     </row>
     <row r="6" spans="1:9" ht="36" customHeight="1">
       <c r="A6" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="G6" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>270</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -7154,7 +7149,7 @@
         <v>0.1185222432255258</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E7" s="17">
         <v>4642722371.0435</v>
@@ -7169,12 +7164,12 @@
         <v>6172360073</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B8" s="15">
         <v>1.5</v>
@@ -7183,7 +7178,7 @@
         <v>0.2252426722271697</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E8" s="17">
         <v>8438016452.3485</v>
@@ -7198,12 +7193,12 @@
         <v>10208037533</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B9" s="15">
         <v>2</v>
@@ -7212,7 +7207,7 @@
         <v>0.3458049896687106</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E9" s="17">
         <v>12604808446.543</v>
@@ -7227,7 +7222,7 @@
         <v>14481981196</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -7271,7 +7266,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7282,7 +7277,7 @@
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7325,7 +7320,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -7336,24 +7331,24 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>85</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B8" s="16">
         <v>0.9709986952715982</v>
@@ -7370,7 +7365,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B9" s="16">
         <v>0.3850957535387177</v>
@@ -7404,7 +7399,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B11" s="16">
         <v>0</v>
@@ -7421,7 +7416,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -7432,24 +7427,24 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>85</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B16" s="16">
         <v>0.9654366988293523</v>
@@ -7466,7 +7461,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B17" s="16">
         <v>0.3812351543942993</v>
@@ -7500,7 +7495,7 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B19" s="16">
         <v>0</v>
@@ -7517,7 +7512,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -7528,24 +7523,24 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>85</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B24" s="16">
         <v>0.9745822850138701</v>
@@ -7562,7 +7557,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B25" s="16">
         <v>0.3651685393258427</v>
@@ -7596,7 +7591,7 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B27" s="16">
         <v>0</v>
@@ -7613,7 +7608,7 @@
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -7624,24 +7619,24 @@
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>85</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B32" s="16">
         <v>0.9877187595947191</v>
@@ -7658,7 +7653,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B33" s="16">
         <v>0.443609022556391</v>
@@ -7692,7 +7687,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B35" s="16">
         <v>0</v>
@@ -7709,7 +7704,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -7720,24 +7715,24 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>85</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B40" s="16">
         <v>0.9848308051341891</v>
@@ -7754,7 +7749,7 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B41" s="16">
         <v>0.5686274509803921</v>
@@ -7788,7 +7783,7 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B43" s="16">
         <v>0</v>
@@ -7895,13 +7890,13 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B2" s="2"/>
     </row>
@@ -7934,66 +7929,66 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>286</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="21" customHeight="1">
       <c r="A7" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>288</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="21" customHeight="1">
       <c r="A8" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>290</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="21" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="21" customHeight="1">
       <c r="A10" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>293</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="21" customHeight="1">
       <c r="A11" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>295</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="21" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="21" customHeight="1">
       <c r="A13" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>298</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="21" customHeight="1">
@@ -8001,55 +7996,55 @@
         <v>88</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="36" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="36" customHeight="1">
       <c r="A16" s="13" t="s">
+        <v>301</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>302</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="36" customHeight="1">
       <c r="A17" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>304</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="36" customHeight="1">
       <c r="A18" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>306</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>308</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1">
       <c r="A21" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="B21" s="14" t="s">
         <v>310</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" customHeight="1">
@@ -8057,7 +8052,7 @@
         <v>32</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
@@ -8065,7 +8060,7 @@
         <v>45</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" customHeight="1">
@@ -8073,7 +8068,7 @@
         <v>46</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" customHeight="1">
@@ -8081,7 +8076,7 @@
         <v>47</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="30" customHeight="1">
@@ -8089,7 +8084,7 @@
         <v>48</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>